<commit_message>
Fix e2eTemplateDownloads.mjs's hardcoded channel count for the 5th marketplace
The sales-import modal's "offers every channel" check asserted exactly
5 template links (4 marketplaces + combined) — now 6 with Temu added.
Also added SALES_TEMU_TEMPLATE.xlsx to the set of expected per-channel
downloads on the Sales Report menu. Re-running in the background to
confirm.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/batch-vs-marketplace/downloaded-sales-report.xlsx
+++ b/e2e-screenshots/batch-vs-marketplace/downloaded-sales-report.xlsx
@@ -10,13 +10,14 @@
     <sheet sheetId="4" name="BM" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="EBAY" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="ONBUY" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="TEMU" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="282">
   <si>
     <t>Sales Report — Audit Summary</t>
   </si>
@@ -64,6 +65,9 @@
   </si>
   <si>
     <t>ONBUY</t>
+  </si>
+  <si>
+    <t>TEMU</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -1269,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1458,42 +1462,66 @@
         <v>18.55</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="4">
         <v>101</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C10" s="4">
         <v>0</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D10" s="4">
         <v>0</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E10" s="4">
         <v>0</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F10" s="5">
         <v>4786.51</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G10" s="5">
         <v>0</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H10" s="5">
         <v>4786.51</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I10" s="5">
         <v>14.49</v>
       </c>
     </row>
-    <row r="11" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1515,6 +1543,11 @@
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1543,57 +1576,57 @@
   <sheetData>
     <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1609,85 +1642,85 @@
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1" t="s">
+        <v>44</v>
+      </c>
+      <c r="N1" t="s">
+        <v>45</v>
+      </c>
+      <c r="O1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>47</v>
+      </c>
+      <c r="R1" t="s">
+        <v>48</v>
+      </c>
+      <c r="S1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T1" t="s">
+        <v>50</v>
+      </c>
+      <c r="U1" t="s">
+        <v>51</v>
+      </c>
+      <c r="V1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="X1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" t="s">
-        <v>40</v>
-      </c>
-      <c r="K1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L1" t="s">
-        <v>42</v>
-      </c>
-      <c r="M1" t="s">
-        <v>43</v>
-      </c>
-      <c r="N1" t="s">
-        <v>44</v>
-      </c>
-      <c r="O1" t="s">
-        <v>35</v>
-      </c>
-      <c r="P1" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>46</v>
-      </c>
-      <c r="R1" t="s">
-        <v>47</v>
-      </c>
-      <c r="S1" t="s">
-        <v>48</v>
-      </c>
-      <c r="T1" t="s">
-        <v>49</v>
-      </c>
-      <c r="U1" t="s">
-        <v>50</v>
-      </c>
-      <c r="V1" t="s">
-        <v>36</v>
-      </c>
-      <c r="W1" t="s">
-        <v>24</v>
-      </c>
-      <c r="X1" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>30</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>31</v>
-      </c>
       <c r="AA1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AB1" t="s">
         <v>10</v>
@@ -1698,16 +1731,16 @@
         <v>46227.5</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -1769,16 +1802,16 @@
         <v>46224.5</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -1840,16 +1873,16 @@
         <v>46224.5</v>
       </c>
       <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" t="s">
         <v>60</v>
-      </c>
-      <c r="C4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E4" t="s">
-        <v>59</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1911,16 +1944,16 @@
         <v>46224.5</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1982,16 +2015,16 @@
         <v>46224.5</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -2053,16 +2086,16 @@
         <v>46220.5</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -2124,16 +2157,16 @@
         <v>46220.5</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -2195,16 +2228,16 @@
         <v>46220.5</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -2266,16 +2299,16 @@
         <v>46220.5</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -2337,16 +2370,16 @@
         <v>46216.5</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -2408,16 +2441,16 @@
         <v>46216.5</v>
       </c>
       <c r="B12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -2479,16 +2512,16 @@
         <v>46216.5</v>
       </c>
       <c r="B13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -2550,16 +2583,16 @@
         <v>46216.5</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -2621,16 +2654,16 @@
         <v>46212.5</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -2692,16 +2725,16 @@
         <v>46212.5</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -2763,16 +2796,16 @@
         <v>46212.5</v>
       </c>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F17">
         <v>1</v>
@@ -2834,16 +2867,16 @@
         <v>46212.5</v>
       </c>
       <c r="B18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -2905,16 +2938,16 @@
         <v>46208.5</v>
       </c>
       <c r="B19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -2976,16 +3009,16 @@
         <v>46208.5</v>
       </c>
       <c r="B20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E20" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -3047,16 +3080,16 @@
         <v>46208.5</v>
       </c>
       <c r="B21" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C21" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F21">
         <v>1</v>
@@ -3118,16 +3151,16 @@
         <v>46208.5</v>
       </c>
       <c r="B22" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F22">
         <v>1</v>
@@ -3189,16 +3222,16 @@
         <v>46204.5</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -3260,16 +3293,16 @@
         <v>46204.5</v>
       </c>
       <c r="B24" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -3331,16 +3364,16 @@
         <v>46204.5</v>
       </c>
       <c r="B25" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C25" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -3402,16 +3435,16 @@
         <v>46204.5</v>
       </c>
       <c r="B26" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C26" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F26">
         <v>1</v>
@@ -3473,16 +3506,16 @@
         <v>46204.5</v>
       </c>
       <c r="B27" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E27" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F27">
         <v>1</v>
@@ -3541,7 +3574,7 @@
     </row>
     <row r="28" spans="1:28" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -3620,76 +3653,76 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L1" t="s">
+        <v>116</v>
+      </c>
+      <c r="M1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" t="s">
+        <v>46</v>
+      </c>
+      <c r="O1" t="s">
+        <v>47</v>
+      </c>
+      <c r="P1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>50</v>
+      </c>
+      <c r="R1" t="s">
+        <v>51</v>
+      </c>
+      <c r="S1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="U1" t="s">
+        <v>30</v>
+      </c>
+      <c r="V1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" t="s">
-        <v>40</v>
-      </c>
-      <c r="K1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L1" t="s">
-        <v>115</v>
-      </c>
-      <c r="M1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N1" t="s">
-        <v>45</v>
-      </c>
-      <c r="O1" t="s">
-        <v>46</v>
-      </c>
-      <c r="P1" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>49</v>
-      </c>
-      <c r="R1" t="s">
-        <v>50</v>
-      </c>
-      <c r="S1" t="s">
-        <v>36</v>
-      </c>
-      <c r="T1" t="s">
-        <v>24</v>
-      </c>
-      <c r="U1" t="s">
-        <v>29</v>
-      </c>
-      <c r="V1" t="s">
-        <v>30</v>
-      </c>
-      <c r="W1" t="s">
-        <v>31</v>
-      </c>
       <c r="X1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y1" t="s">
         <v>10</v>
@@ -3700,16 +3733,16 @@
         <v>46225.5</v>
       </c>
       <c r="B2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -3762,16 +3795,16 @@
         <v>46225.5</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -3824,16 +3857,16 @@
         <v>46225.5</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -3886,16 +3919,16 @@
         <v>46225.5</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -3948,16 +3981,16 @@
         <v>46221.5</v>
       </c>
       <c r="B6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -4010,16 +4043,16 @@
         <v>46221.5</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -4072,16 +4105,16 @@
         <v>46221.5</v>
       </c>
       <c r="B8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -4134,16 +4167,16 @@
         <v>46221.5</v>
       </c>
       <c r="B9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -4196,16 +4229,16 @@
         <v>46217.5</v>
       </c>
       <c r="B10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -4258,16 +4291,16 @@
         <v>46217.5</v>
       </c>
       <c r="B11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -4320,16 +4353,16 @@
         <v>46217.5</v>
       </c>
       <c r="B12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -4382,16 +4415,16 @@
         <v>46217.5</v>
       </c>
       <c r="B13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -4444,16 +4477,16 @@
         <v>46213.5</v>
       </c>
       <c r="B14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -4506,16 +4539,16 @@
         <v>46213.5</v>
       </c>
       <c r="B15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -4568,16 +4601,16 @@
         <v>46213.5</v>
       </c>
       <c r="B16" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -4630,16 +4663,16 @@
         <v>46213.5</v>
       </c>
       <c r="B17" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F17">
         <v>1</v>
@@ -4692,16 +4725,16 @@
         <v>46209.5</v>
       </c>
       <c r="B18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -4754,16 +4787,16 @@
         <v>46209.5</v>
       </c>
       <c r="B19" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C19" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -4816,16 +4849,16 @@
         <v>46209.5</v>
       </c>
       <c r="B20" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -4878,16 +4911,16 @@
         <v>46209.5</v>
       </c>
       <c r="B21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E21" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F21">
         <v>1</v>
@@ -4940,16 +4973,16 @@
         <v>46205.5</v>
       </c>
       <c r="B22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F22">
         <v>1</v>
@@ -5002,16 +5035,16 @@
         <v>46205.5</v>
       </c>
       <c r="B23" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -5064,16 +5097,16 @@
         <v>46205.5</v>
       </c>
       <c r="B24" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -5126,16 +5159,16 @@
         <v>46205.5</v>
       </c>
       <c r="B25" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C25" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -5188,16 +5221,16 @@
         <v>46205.5</v>
       </c>
       <c r="B26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C26" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F26">
         <v>1</v>
@@ -5247,7 +5280,7 @@
     </row>
     <row r="27" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -5317,94 +5350,94 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>161</v>
+      </c>
+      <c r="G1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M1" t="s">
+        <v>163</v>
+      </c>
+      <c r="N1" t="s">
+        <v>164</v>
+      </c>
+      <c r="O1" t="s">
+        <v>165</v>
+      </c>
+      <c r="P1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>46</v>
+      </c>
+      <c r="R1" t="s">
+        <v>166</v>
+      </c>
+      <c r="S1" t="s">
+        <v>167</v>
+      </c>
+      <c r="T1" t="s">
+        <v>47</v>
+      </c>
+      <c r="U1" t="s">
+        <v>48</v>
+      </c>
+      <c r="V1" t="s">
+        <v>49</v>
+      </c>
+      <c r="W1" t="s">
+        <v>50</v>
+      </c>
+      <c r="X1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" t="s">
-        <v>160</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="AA1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" t="s">
-        <v>40</v>
-      </c>
-      <c r="K1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L1" t="s">
-        <v>161</v>
-      </c>
-      <c r="M1" t="s">
-        <v>162</v>
-      </c>
-      <c r="N1" t="s">
-        <v>163</v>
-      </c>
-      <c r="O1" t="s">
-        <v>164</v>
-      </c>
-      <c r="P1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>45</v>
-      </c>
-      <c r="R1" t="s">
-        <v>165</v>
-      </c>
-      <c r="S1" t="s">
-        <v>166</v>
-      </c>
-      <c r="T1" t="s">
-        <v>46</v>
-      </c>
-      <c r="U1" t="s">
-        <v>47</v>
-      </c>
-      <c r="V1" t="s">
-        <v>48</v>
-      </c>
-      <c r="W1" t="s">
-        <v>49</v>
-      </c>
-      <c r="X1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>31</v>
-      </c>
       <c r="AD1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AE1" t="s">
         <v>10</v>
@@ -5415,16 +5448,16 @@
         <v>46226.5</v>
       </c>
       <c r="B2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -5495,16 +5528,16 @@
         <v>46226.5</v>
       </c>
       <c r="B3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -5575,16 +5608,16 @@
         <v>46226.5</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -5655,16 +5688,16 @@
         <v>46226.5</v>
       </c>
       <c r="B5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -5735,16 +5768,16 @@
         <v>46222.5</v>
       </c>
       <c r="B6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -5815,16 +5848,16 @@
         <v>46222.5</v>
       </c>
       <c r="B7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -5895,16 +5928,16 @@
         <v>46222.5</v>
       </c>
       <c r="B8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -5975,16 +6008,16 @@
         <v>46222.5</v>
       </c>
       <c r="B9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -6055,16 +6088,16 @@
         <v>46218.5</v>
       </c>
       <c r="B10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -6135,16 +6168,16 @@
         <v>46218.5</v>
       </c>
       <c r="B11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -6215,16 +6248,16 @@
         <v>46218.5</v>
       </c>
       <c r="B12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -6295,16 +6328,16 @@
         <v>46218.5</v>
       </c>
       <c r="B13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -6375,16 +6408,16 @@
         <v>46214.5</v>
       </c>
       <c r="B14" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -6455,16 +6488,16 @@
         <v>46214.5</v>
       </c>
       <c r="B15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -6535,16 +6568,16 @@
         <v>46214.5</v>
       </c>
       <c r="B16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -6615,16 +6648,16 @@
         <v>46214.5</v>
       </c>
       <c r="B17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F17">
         <v>1</v>
@@ -6695,16 +6728,16 @@
         <v>46210.5</v>
       </c>
       <c r="B18" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -6775,16 +6808,16 @@
         <v>46210.5</v>
       </c>
       <c r="B19" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -6855,16 +6888,16 @@
         <v>46210.5</v>
       </c>
       <c r="B20" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E20" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -6935,16 +6968,16 @@
         <v>46210.5</v>
       </c>
       <c r="B21" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F21">
         <v>1</v>
@@ -7015,16 +7048,16 @@
         <v>46206.5</v>
       </c>
       <c r="B22" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F22">
         <v>1</v>
@@ -7095,16 +7128,16 @@
         <v>46206.5</v>
       </c>
       <c r="B23" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E23" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -7175,16 +7208,16 @@
         <v>46206.5</v>
       </c>
       <c r="B24" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -7255,16 +7288,16 @@
         <v>46206.5</v>
       </c>
       <c r="B25" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C25" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -7335,16 +7368,16 @@
         <v>46206.5</v>
       </c>
       <c r="B26" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C26" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E26" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F26">
         <v>1</v>
@@ -7412,7 +7445,7 @@
     </row>
     <row r="27" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -7500,76 +7533,76 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" t="s">
+        <v>224</v>
+      </c>
+      <c r="L1" t="s">
+        <v>36</v>
+      </c>
+      <c r="M1" t="s">
+        <v>46</v>
+      </c>
+      <c r="N1" t="s">
+        <v>47</v>
+      </c>
+      <c r="O1" t="s">
+        <v>48</v>
+      </c>
+      <c r="P1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>50</v>
+      </c>
+      <c r="R1" t="s">
+        <v>51</v>
+      </c>
+      <c r="S1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="U1" t="s">
+        <v>30</v>
+      </c>
+      <c r="V1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" t="s">
         <v>32</v>
       </c>
-      <c r="G1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
-      </c>
-      <c r="K1" t="s">
-        <v>223</v>
-      </c>
-      <c r="L1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M1" t="s">
-        <v>45</v>
-      </c>
-      <c r="N1" t="s">
-        <v>46</v>
-      </c>
-      <c r="O1" t="s">
-        <v>47</v>
-      </c>
-      <c r="P1" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>49</v>
-      </c>
-      <c r="R1" t="s">
-        <v>50</v>
-      </c>
-      <c r="S1" t="s">
-        <v>36</v>
-      </c>
-      <c r="T1" t="s">
-        <v>24</v>
-      </c>
-      <c r="U1" t="s">
-        <v>29</v>
-      </c>
-      <c r="V1" t="s">
-        <v>30</v>
-      </c>
-      <c r="W1" t="s">
-        <v>31</v>
-      </c>
       <c r="X1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y1" t="s">
         <v>10</v>
@@ -7580,16 +7613,16 @@
         <v>46227.5</v>
       </c>
       <c r="B2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F2" s="3">
         <v>264.82</v>
@@ -7642,16 +7675,16 @@
         <v>46227.5</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F3" s="3">
         <v>256.93</v>
@@ -7704,16 +7737,16 @@
         <v>46227.5</v>
       </c>
       <c r="B4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F4" s="3">
         <v>276.86</v>
@@ -7766,16 +7799,16 @@
         <v>46227.5</v>
       </c>
       <c r="B5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F5" s="3">
         <v>293.74</v>
@@ -7828,16 +7861,16 @@
         <v>46223.5</v>
       </c>
       <c r="B6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F6" s="3">
         <v>500.16</v>
@@ -7890,16 +7923,16 @@
         <v>46223.5</v>
       </c>
       <c r="B7" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F7" s="3">
         <v>500.85</v>
@@ -7952,16 +7985,16 @@
         <v>46223.5</v>
       </c>
       <c r="B8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F8" s="3">
         <v>529.23</v>
@@ -8014,16 +8047,16 @@
         <v>46223.5</v>
       </c>
       <c r="B9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F9" s="3">
         <v>530.25</v>
@@ -8076,16 +8109,16 @@
         <v>46219.5</v>
       </c>
       <c r="B10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F10" s="3">
         <v>275.49</v>
@@ -8138,16 +8171,16 @@
         <v>46219.5</v>
       </c>
       <c r="B11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F11" s="3">
         <v>287.02</v>
@@ -8200,16 +8233,16 @@
         <v>46219.5</v>
       </c>
       <c r="B12" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C12" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F12" s="3">
         <v>268.59</v>
@@ -8262,16 +8295,16 @@
         <v>46219.5</v>
       </c>
       <c r="B13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C13" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F13" s="3">
         <v>280.37</v>
@@ -8324,16 +8357,16 @@
         <v>46215.5</v>
       </c>
       <c r="B14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F14" s="3">
         <v>511.35</v>
@@ -8386,16 +8419,16 @@
         <v>46215.5</v>
       </c>
       <c r="B15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F15" s="3">
         <v>507.95</v>
@@ -8448,16 +8481,16 @@
         <v>46215.5</v>
       </c>
       <c r="B16" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F16" s="3">
         <v>495.98</v>
@@ -8510,16 +8543,16 @@
         <v>46215.5</v>
       </c>
       <c r="B17" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F17" s="3">
         <v>514.23</v>
@@ -8572,16 +8605,16 @@
         <v>46211.5</v>
       </c>
       <c r="B18" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F18" s="3">
         <v>262.14</v>
@@ -8634,16 +8667,16 @@
         <v>46211.5</v>
       </c>
       <c r="B19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C19" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F19" s="3">
         <v>267</v>
@@ -8696,16 +8729,16 @@
         <v>46211.5</v>
       </c>
       <c r="B20" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C20" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E20" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F20" s="3">
         <v>290.37</v>
@@ -8758,16 +8791,16 @@
         <v>46211.5</v>
       </c>
       <c r="B21" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C21" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F21" s="3">
         <v>260.29</v>
@@ -8820,16 +8853,16 @@
         <v>46207.5</v>
       </c>
       <c r="B22" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F22" s="3">
         <v>501.14</v>
@@ -8882,16 +8915,16 @@
         <v>46207.5</v>
       </c>
       <c r="B23" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E23" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F23" s="3">
         <v>533.2</v>
@@ -8944,16 +8977,16 @@
         <v>46207.5</v>
       </c>
       <c r="B24" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F24" s="3">
         <v>499.91</v>
@@ -9006,16 +9039,16 @@
         <v>46207.5</v>
       </c>
       <c r="B25" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F25" s="3">
         <v>535.83</v>
@@ -9068,16 +9101,16 @@
         <v>46207.5</v>
       </c>
       <c r="B26" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F26" s="3">
         <v>517.1</v>
@@ -9127,7 +9160,7 @@
     </row>
     <row r="27" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -9188,4 +9221,101 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AB1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1" t="s">
+        <v>44</v>
+      </c>
+      <c r="N1" t="s">
+        <v>45</v>
+      </c>
+      <c r="O1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>47</v>
+      </c>
+      <c r="R1" t="s">
+        <v>48</v>
+      </c>
+      <c r="S1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T1" t="s">
+        <v>50</v>
+      </c>
+      <c r="U1" t="s">
+        <v>51</v>
+      </c>
+      <c r="V1" t="s">
+        <v>37</v>
+      </c>
+      <c r="W1" t="s">
+        <v>25</v>
+      </c>
+      <c r="X1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh E2E evidence screenshots; clarify accessory test docs
Re-ran all 17 Playwright suites fresh (311/311 checks) to regenerate
current, reproducible screenshots for the client evidence PDF — these
now reflect the corrected Temu formulas and the new AccessoryStock
feature rather than pre-fix state.

Also updates accessoryIntake.test.ts's docstring: an earlier decision
in this same project correctly kept identifier-less accessories out of
the per-unit master-file importer (that importer still rejects them,
unchanged). Clarifies that the "different stock model" the comment
predicted would be needed now exists as AccessoryStock, reached through
a separate Add Stock tab — no functional change, no contradiction with
that earlier decision.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/batch-vs-marketplace/downloaded-sales-report.xlsx
+++ b/e2e-screenshots/batch-vs-marketplace/downloaded-sales-report.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="283">
   <si>
     <t>Sales Report — Audit Summary</t>
   </si>
@@ -863,6 +863,9 @@
   </si>
   <si>
     <t>350100007911081</t>
+  </si>
+  <si>
+    <t>Commission VAT</t>
   </si>
 </sst>
 </file>
@@ -9225,10 +9228,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>39</v>
       </c>
@@ -9263,54 +9266,48 @@
         <v>42</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>282</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O1" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="P1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="Q1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="R1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="S1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="T1" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="U1" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="V1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="W1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="X1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="Y1" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="Z1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB1" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>